<commit_message>
working on figure 3.1.1
</commit_message>
<xml_diff>
--- a/IP_Absorption.xlsx
+++ b/IP_Absorption.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nuwildcat-my.sharepoint.com/personal/stn424_ads_northwestern_edu/Documents/Collaborations/Proposals/GO-Barrier, TFMI Proposals with Tim Wei/URAP_2023-10/Shared/Lanning, Mackenzie/Absorption Data/Fall 2025/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nuwildcat-my.sharepoint.com/personal/stn424_ads_northwestern_edu/Documents/Collaborations/Proposals/GO-Barrier, TFMI Proposals with Tim Wei/URAP_2023-10/Shared/Lanning, Mackenzie/graphene-oxide-paper-coatings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="272" documentId="8_{D2BF99F2-6939-1445-9333-69AF606EB5C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CEC24DE-3DFB-1743-B271-E02198743697}"/>
+  <xr:revisionPtr revIDLastSave="277" documentId="8_{D2BF99F2-6939-1445-9333-69AF606EB5C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBE1EDA3-0506-C34B-9FD5-F9BFC4B63900}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="15620" windowHeight="17180" activeTab="2" xr2:uid="{E0E81384-8338-6A40-B1D6-6AC1A920927D}"/>
   </bookViews>
@@ -220,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -301,13 +301,14 @@
     </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15159,24 +15160,24 @@
       <c r="P44" s="4"/>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A45" s="30" t="s">
+      <c r="A45" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="B45" s="30"/>
-      <c r="C45" s="30"/>
-      <c r="D45" s="30"/>
-      <c r="E45" s="30"/>
-      <c r="F45" s="30"/>
-      <c r="G45" s="30"/>
-      <c r="H45" s="30"/>
-      <c r="I45" s="30"/>
-      <c r="J45" s="30"/>
-      <c r="K45" s="30"/>
-      <c r="L45" s="30"/>
-      <c r="M45" s="30"/>
-      <c r="N45" s="30"/>
-      <c r="O45" s="30"/>
-      <c r="P45" s="30"/>
+      <c r="B45" s="31"/>
+      <c r="C45" s="31"/>
+      <c r="D45" s="31"/>
+      <c r="E45" s="31"/>
+      <c r="F45" s="31"/>
+      <c r="G45" s="31"/>
+      <c r="H45" s="31"/>
+      <c r="I45" s="31"/>
+      <c r="J45" s="31"/>
+      <c r="K45" s="31"/>
+      <c r="L45" s="31"/>
+      <c r="M45" s="31"/>
+      <c r="N45" s="31"/>
+      <c r="O45" s="31"/>
+      <c r="P45" s="31"/>
     </row>
     <row r="46" spans="1:16" ht="51" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
@@ -18283,13 +18284,13 @@
       <c r="F1" s="2"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
       <c r="F2" s="1"/>
     </row>
     <row r="3" spans="1:8" ht="51" x14ac:dyDescent="0.2">
@@ -19341,13 +19342,13 @@
       <c r="F52" s="4"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A53" s="30" t="s">
+      <c r="A53" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="B53" s="30"/>
-      <c r="C53" s="30"/>
-      <c r="D53" s="30"/>
-      <c r="E53" s="30"/>
+      <c r="B53" s="31"/>
+      <c r="C53" s="31"/>
+      <c r="D53" s="31"/>
+      <c r="E53" s="31"/>
       <c r="F53" s="1"/>
     </row>
     <row r="54" spans="1:8" ht="51" x14ac:dyDescent="0.2">
@@ -22055,14 +22056,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37BD9F41-A594-794A-B79F-91E3A34AD959}">
-  <dimension ref="A1:D211"/>
+  <dimension ref="A1:F211"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="12.6640625" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="26" t="s">
         <v>22</v>
       </c>
@@ -22076,7 +22077,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="27">
         <v>0</v>
       </c>
@@ -22086,11 +22087,11 @@
       <c r="C2" s="19">
         <v>0.85499999999999998</v>
       </c>
-      <c r="D2" s="32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D2" s="30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="27">
         <v>0</v>
       </c>
@@ -22100,11 +22101,11 @@
       <c r="C3" s="19">
         <v>0.84399999999999997</v>
       </c>
-      <c r="D3" s="32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D3" s="30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="27">
         <v>0</v>
       </c>
@@ -22114,11 +22115,11 @@
       <c r="C4" s="19">
         <v>0.85</v>
       </c>
-      <c r="D4" s="32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D4" s="30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="27">
         <v>0</v>
       </c>
@@ -22128,11 +22129,11 @@
       <c r="C5" s="19">
         <v>0.84199999999999997</v>
       </c>
-      <c r="D5" s="32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D5" s="30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="27">
         <v>0</v>
       </c>
@@ -22142,11 +22143,12 @@
       <c r="C6" s="19">
         <v>0.85199999999999998</v>
       </c>
-      <c r="D6" s="32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D6" s="30">
+        <v>0</v>
+      </c>
+      <c r="F6" s="33"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="27">
         <v>10</v>
       </c>
@@ -22156,11 +22158,11 @@
       <c r="C7" s="19">
         <v>0.995</v>
       </c>
-      <c r="D7" s="32">
+      <c r="D7" s="30">
         <v>4.3400086800173604E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="27">
         <v>10</v>
       </c>
@@ -22170,11 +22172,11 @@
       <c r="C8" s="19">
         <v>0.97799999999999998</v>
       </c>
-      <c r="D8" s="32">
+      <c r="D8" s="30">
         <v>4.1540083080166155E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="27">
         <v>10</v>
       </c>
@@ -22184,11 +22186,11 @@
       <c r="C9" s="19">
         <v>0.98899999999999999</v>
       </c>
-      <c r="D9" s="32">
+      <c r="D9" s="30">
         <v>4.3090086180172359E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="27">
         <v>10</v>
       </c>
@@ -22198,11 +22200,11 @@
       <c r="C10" s="19">
         <v>0.98199999999999998</v>
       </c>
-      <c r="D10" s="32">
+      <c r="D10" s="30">
         <v>4.3400086800173604E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="27">
         <v>10</v>
       </c>
@@ -22212,11 +22214,11 @@
       <c r="C11" s="19">
         <v>0.99199999999999999</v>
       </c>
-      <c r="D11" s="32">
+      <c r="D11" s="30">
         <v>4.3400086800173604E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="27">
         <v>20</v>
       </c>
@@ -22226,11 +22228,11 @@
       <c r="C12" s="19">
         <v>1.048</v>
       </c>
-      <c r="D12" s="32">
+      <c r="D12" s="30">
         <v>5.9830119660239335E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="27">
         <v>20</v>
       </c>
@@ -22240,11 +22242,11 @@
       <c r="C13" s="19">
         <v>1.03</v>
       </c>
-      <c r="D13" s="32">
+      <c r="D13" s="30">
         <v>5.7660115320230651E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="27">
         <v>20</v>
       </c>
@@ -22254,11 +22256,11 @@
       <c r="C14" s="19">
         <v>1.0429999999999999</v>
       </c>
-      <c r="D14" s="32">
+      <c r="D14" s="30">
         <v>5.98301196602393E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="27">
         <v>20</v>
       </c>
@@ -22268,11 +22270,11 @@
       <c r="C15" s="19">
         <v>1.0249999999999999</v>
       </c>
-      <c r="D15" s="32">
+      <c r="D15" s="30">
         <v>5.67301134602269E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="27">
         <v>20</v>
       </c>
@@ -22282,7 +22284,7 @@
       <c r="C16" s="19">
         <v>1.0389999999999999</v>
       </c>
-      <c r="D16" s="32">
+      <c r="D16" s="30">
         <v>5.797011594023186E-3</v>
       </c>
     </row>
@@ -22296,7 +22298,7 @@
       <c r="C17" s="19">
         <v>1.0780000000000001</v>
       </c>
-      <c r="D17" s="32">
+      <c r="D17" s="30">
         <v>6.9130138260276542E-3</v>
       </c>
     </row>
@@ -22310,7 +22312,7 @@
       <c r="C18" s="19">
         <v>1.0589999999999999</v>
       </c>
-      <c r="D18" s="32">
+      <c r="D18" s="30">
         <v>6.6650133300266588E-3</v>
       </c>
     </row>
@@ -22324,7 +22326,7 @@
       <c r="C19" s="19">
         <v>1.069</v>
       </c>
-      <c r="D19" s="32">
+      <c r="D19" s="30">
         <v>6.7890135780271548E-3</v>
       </c>
     </row>
@@ -22338,7 +22340,7 @@
       <c r="C20" s="19">
         <v>1.048</v>
       </c>
-      <c r="D20" s="32">
+      <c r="D20" s="30">
         <v>6.3860127720255459E-3</v>
       </c>
     </row>
@@ -22352,7 +22354,7 @@
       <c r="C21" s="19">
         <v>1.0640000000000001</v>
       </c>
-      <c r="D21" s="32">
+      <c r="D21" s="30">
         <v>6.5720131440262898E-3</v>
       </c>
     </row>
@@ -22366,7 +22368,7 @@
       <c r="C22" s="19">
         <v>1.099</v>
       </c>
-      <c r="D22" s="32">
+      <c r="D22" s="30">
         <v>7.5640151280302551E-3</v>
       </c>
     </row>
@@ -22380,7 +22382,7 @@
       <c r="C23" s="19">
         <v>1.087</v>
       </c>
-      <c r="D23" s="32">
+      <c r="D23" s="30">
         <v>7.5330150660301316E-3</v>
       </c>
     </row>
@@ -22394,7 +22396,7 @@
       <c r="C24" s="19">
         <v>1.0980000000000001</v>
       </c>
-      <c r="D24" s="32">
+      <c r="D24" s="30">
         <v>7.6880153760307546E-3</v>
       </c>
     </row>
@@ -22408,7 +22410,7 @@
       <c r="C25" s="19">
         <v>1.073</v>
       </c>
-      <c r="D25" s="32">
+      <c r="D25" s="30">
         <v>7.1610143220286427E-3</v>
       </c>
     </row>
@@ -22422,7 +22424,7 @@
       <c r="C26" s="19">
         <v>1.0940000000000001</v>
       </c>
-      <c r="D26" s="32">
+      <c r="D26" s="30">
         <v>7.5020150040300106E-3</v>
       </c>
     </row>
@@ -22436,7 +22438,7 @@
       <c r="C27" s="19">
         <v>1.1200000000000001</v>
       </c>
-      <c r="D27" s="32">
+      <c r="D27" s="30">
         <v>8.2150164300328638E-3</v>
       </c>
     </row>
@@ -22450,7 +22452,7 @@
       <c r="C28" s="19">
         <v>1.1060000000000001</v>
       </c>
-      <c r="D28" s="32">
+      <c r="D28" s="30">
         <v>8.1220162440324914E-3</v>
       </c>
     </row>
@@ -22464,7 +22466,7 @@
       <c r="C29" s="19">
         <v>1.1279999999999999</v>
       </c>
-      <c r="D29" s="32">
+      <c r="D29" s="30">
         <v>8.6180172360344684E-3</v>
       </c>
     </row>
@@ -22478,7 +22480,7 @@
       <c r="C30" s="19">
         <v>1.095</v>
       </c>
-      <c r="D30" s="32">
+      <c r="D30" s="30">
         <v>7.8430156860313707E-3</v>
       </c>
     </row>
@@ -22492,7 +22494,7 @@
       <c r="C31" s="19">
         <v>1.1140000000000001</v>
       </c>
-      <c r="D31" s="32">
+      <c r="D31" s="30">
         <v>8.1220162440324914E-3</v>
       </c>
     </row>
@@ -22506,7 +22508,7 @@
       <c r="C32" s="19">
         <v>1.155</v>
       </c>
-      <c r="D32" s="32">
+      <c r="D32" s="30">
         <v>9.3000186000372007E-3</v>
       </c>
     </row>
@@ -22520,7 +22522,7 @@
       <c r="C33" s="19">
         <v>1.135</v>
       </c>
-      <c r="D33" s="32">
+      <c r="D33" s="30">
         <v>9.0210180420360851E-3</v>
       </c>
     </row>
@@ -22534,7 +22536,7 @@
       <c r="C34" s="19">
         <v>1.157</v>
       </c>
-      <c r="D34" s="32">
+      <c r="D34" s="30">
         <v>9.5170190340380691E-3</v>
       </c>
     </row>
@@ -22548,7 +22550,7 @@
       <c r="C35" s="19">
         <v>1.1080000000000001</v>
       </c>
-      <c r="D35" s="32">
+      <c r="D35" s="30">
         <v>8.2460164920329874E-3</v>
       </c>
     </row>
@@ -22562,7 +22564,7 @@
       <c r="C36" s="19">
         <v>1.1259999999999999</v>
       </c>
-      <c r="D36" s="32">
+      <c r="D36" s="30">
         <v>8.4940169880339724E-3</v>
       </c>
     </row>
@@ -22576,7 +22578,7 @@
       <c r="C37" s="19">
         <v>0.81200000000000006</v>
       </c>
-      <c r="D37" s="32">
+      <c r="D37" s="30">
         <v>0</v>
       </c>
     </row>
@@ -22590,7 +22592,7 @@
       <c r="C38" s="19">
         <v>0.82799999999999996</v>
       </c>
-      <c r="D38" s="32">
+      <c r="D38" s="30">
         <v>0</v>
       </c>
     </row>
@@ -22604,7 +22606,7 @@
       <c r="C39" s="19">
         <v>0.80900000000000005</v>
       </c>
-      <c r="D39" s="32">
+      <c r="D39" s="30">
         <v>0</v>
       </c>
     </row>
@@ -22618,7 +22620,7 @@
       <c r="C40" s="19">
         <v>0.80900000000000005</v>
       </c>
-      <c r="D40" s="32">
+      <c r="D40" s="30">
         <v>0</v>
       </c>
     </row>
@@ -22632,7 +22634,7 @@
       <c r="C41" s="19">
         <v>0.84</v>
       </c>
-      <c r="D41" s="32">
+      <c r="D41" s="30">
         <v>0</v>
       </c>
     </row>
@@ -22646,7 +22648,7 @@
       <c r="C42" s="19">
         <v>0.97199999999999998</v>
       </c>
-      <c r="D42" s="32">
+      <c r="D42" s="30">
         <v>4.9600099200198368E-3</v>
       </c>
     </row>
@@ -22660,7 +22662,7 @@
       <c r="C43" s="19">
         <v>0.98799999999999999</v>
       </c>
-      <c r="D43" s="32">
+      <c r="D43" s="30">
         <v>4.9600099200198403E-3</v>
       </c>
     </row>
@@ -22674,7 +22676,7 @@
       <c r="C44" s="19">
         <v>0.97899999999999998</v>
       </c>
-      <c r="D44" s="32">
+      <c r="D44" s="30">
         <v>5.2700105400210777E-3</v>
       </c>
     </row>
@@ -22688,7 +22690,7 @@
       <c r="C45" s="19">
         <v>0.97599999999999998</v>
       </c>
-      <c r="D45" s="32">
+      <c r="D45" s="30">
         <v>5.1770103540207052E-3</v>
       </c>
     </row>
@@ -22702,7 +22704,7 @@
       <c r="C46" s="19">
         <v>1.02</v>
       </c>
-      <c r="D46" s="32">
+      <c r="D46" s="30">
         <v>5.5800111600223211E-3</v>
       </c>
     </row>
@@ -22716,7 +22718,7 @@
       <c r="C47" s="19">
         <v>1.0029999999999999</v>
       </c>
-      <c r="D47" s="32">
+      <c r="D47" s="30">
         <v>5.9210118420236785E-3</v>
       </c>
     </row>
@@ -22730,7 +22732,7 @@
       <c r="C48" s="19">
         <v>1.02</v>
       </c>
-      <c r="D48" s="32">
+      <c r="D48" s="30">
         <v>5.952011904023809E-3</v>
       </c>
     </row>
@@ -22744,7 +22746,7 @@
       <c r="C49" s="19">
         <v>1.004</v>
       </c>
-      <c r="D49" s="32">
+      <c r="D49" s="30">
         <v>6.045012090024178E-3</v>
       </c>
     </row>
@@ -22758,7 +22760,7 @@
       <c r="C50" s="19">
         <v>1.006</v>
       </c>
-      <c r="D50" s="32">
+      <c r="D50" s="30">
         <v>6.107012214024426E-3</v>
       </c>
     </row>
@@ -22772,7 +22774,7 @@
       <c r="C51" s="19">
         <v>1.054</v>
       </c>
-      <c r="D51" s="32">
+      <c r="D51" s="30">
         <v>6.6340132680265378E-3</v>
       </c>
     </row>
@@ -22786,7 +22788,7 @@
       <c r="C52" s="19">
         <v>1.0229999999999999</v>
       </c>
-      <c r="D52" s="32">
+      <c r="D52" s="30">
         <v>6.5410130820261593E-3</v>
       </c>
     </row>
@@ -22800,7 +22802,7 @@
       <c r="C53" s="19">
         <v>1.0409999999999999</v>
       </c>
-      <c r="D53" s="32">
+      <c r="D53" s="30">
         <v>6.6030132060264108E-3</v>
       </c>
     </row>
@@ -22814,7 +22816,7 @@
       <c r="C54" s="19">
         <v>1.0309999999999999</v>
       </c>
-      <c r="D54" s="32">
+      <c r="D54" s="30">
         <v>6.8820137640275229E-3</v>
       </c>
     </row>
@@ -22828,7 +22830,7 @@
       <c r="C55" s="19">
         <v>1.0309999999999999</v>
       </c>
-      <c r="D55" s="32">
+      <c r="D55" s="30">
         <v>6.8820137640275229E-3</v>
       </c>
     </row>
@@ -22842,7 +22844,7 @@
       <c r="C56" s="19">
         <v>1.079</v>
       </c>
-      <c r="D56" s="32">
+      <c r="D56" s="30">
         <v>7.4090148180296356E-3</v>
       </c>
     </row>
@@ -22856,7 +22858,7 @@
       <c r="C57" s="19">
         <v>1.0349999999999999</v>
       </c>
-      <c r="D57" s="32">
+      <c r="D57" s="30">
         <v>6.9130138260276473E-3</v>
       </c>
     </row>
@@ -22870,7 +22872,7 @@
       <c r="C58" s="19">
         <v>1.0609999999999999</v>
       </c>
-      <c r="D58" s="32">
+      <c r="D58" s="30">
         <v>7.2230144460288907E-3</v>
       </c>
     </row>
@@ -22884,7 +22886,7 @@
       <c r="C59" s="19">
         <v>1.0509999999999999</v>
       </c>
-      <c r="D59" s="32">
+      <c r="D59" s="30">
         <v>7.5020150040300037E-3</v>
       </c>
     </row>
@@ -22898,7 +22900,7 @@
       <c r="C60" s="19">
         <v>1.0389999999999999</v>
       </c>
-      <c r="D60" s="32">
+      <c r="D60" s="30">
         <v>7.1300142600285157E-3</v>
       </c>
     </row>
@@ -22912,7 +22914,7 @@
       <c r="C61" s="19">
         <v>1.089</v>
       </c>
-      <c r="D61" s="32">
+      <c r="D61" s="30">
         <v>7.7190154380308755E-3</v>
       </c>
     </row>
@@ -22926,7 +22928,7 @@
       <c r="C62" s="19">
         <v>1.052</v>
       </c>
-      <c r="D62" s="32">
+      <c r="D62" s="30">
         <v>7.4400148800297591E-3</v>
       </c>
     </row>
@@ -22940,7 +22942,7 @@
       <c r="C63" s="19">
         <v>1.071</v>
       </c>
-      <c r="D63" s="32">
+      <c r="D63" s="30">
         <v>7.5330150660301316E-3</v>
       </c>
     </row>
@@ -22954,7 +22956,7 @@
       <c r="C64" s="19">
         <v>1.0660000000000001</v>
       </c>
-      <c r="D64" s="32">
+      <c r="D64" s="30">
         <v>7.9670159340318684E-3</v>
       </c>
     </row>
@@ -22968,7 +22970,7 @@
       <c r="C65" s="19">
         <v>1.054</v>
       </c>
-      <c r="D65" s="32">
+      <c r="D65" s="30">
         <v>7.5950151900303796E-3</v>
       </c>
     </row>
@@ -22982,7 +22984,7 @@
       <c r="C66" s="19">
         <v>1.113</v>
       </c>
-      <c r="D66" s="32">
+      <c r="D66" s="30">
         <v>8.4630169260338523E-3</v>
       </c>
     </row>
@@ -22996,7 +22998,7 @@
       <c r="C67" s="19">
         <v>1.0609999999999999</v>
       </c>
-      <c r="D67" s="32">
+      <c r="D67" s="30">
         <v>7.7190154380308721E-3</v>
       </c>
     </row>
@@ -23010,7 +23012,7 @@
       <c r="C68" s="19">
         <v>1.081</v>
       </c>
-      <c r="D68" s="32">
+      <c r="D68" s="30">
         <v>7.8430156860313707E-3</v>
       </c>
     </row>
@@ -23024,7 +23026,7 @@
       <c r="C69" s="19">
         <v>1.0680000000000001</v>
       </c>
-      <c r="D69" s="32">
+      <c r="D69" s="30">
         <v>8.0290160580321155E-3</v>
       </c>
     </row>
@@ -23038,7 +23040,7 @@
       <c r="C70" s="19">
         <v>1.0680000000000001</v>
       </c>
-      <c r="D70" s="32">
+      <c r="D70" s="30">
         <v>8.0290160580321155E-3</v>
       </c>
     </row>
@@ -23052,7 +23054,7 @@
       <c r="C71" s="19">
         <v>1.131</v>
       </c>
-      <c r="D71" s="32">
+      <c r="D71" s="30">
         <v>9.0210180420360851E-3</v>
       </c>
     </row>
@@ -23066,7 +23068,7 @@
       <c r="C72" s="20">
         <v>0.82099999999999995</v>
       </c>
-      <c r="D72" s="32">
+      <c r="D72" s="30">
         <v>0</v>
       </c>
     </row>
@@ -23080,7 +23082,7 @@
       <c r="C73" s="20">
         <v>0.82199999999999995</v>
       </c>
-      <c r="D73" s="32">
+      <c r="D73" s="30">
         <v>0</v>
       </c>
     </row>
@@ -23094,7 +23096,7 @@
       <c r="C74" s="20">
         <v>0.82599999999999996</v>
       </c>
-      <c r="D74" s="32">
+      <c r="D74" s="30">
         <v>0</v>
       </c>
     </row>
@@ -23108,7 +23110,7 @@
       <c r="C75" s="20">
         <v>0.84399999999999997</v>
       </c>
-      <c r="D75" s="32">
+      <c r="D75" s="30">
         <v>0</v>
       </c>
     </row>
@@ -23122,7 +23124,7 @@
       <c r="C76" s="20">
         <v>0.84899999999999998</v>
       </c>
-      <c r="D76" s="32">
+      <c r="D76" s="30">
         <v>0</v>
       </c>
     </row>
@@ -23136,7 +23138,7 @@
       <c r="C77" s="20">
         <v>0.99199999999999999</v>
       </c>
-      <c r="D77" s="32">
+      <c r="D77" s="30">
         <v>5.3010106020212047E-3</v>
       </c>
     </row>
@@ -23150,7 +23152,7 @@
       <c r="C78" s="20">
         <v>0.98499999999999999</v>
       </c>
-      <c r="D78" s="32">
+      <c r="D78" s="30">
         <v>5.0530101060202127E-3</v>
       </c>
     </row>
@@ -23164,7 +23166,7 @@
       <c r="C79" s="20">
         <v>0.98899999999999999</v>
       </c>
-      <c r="D79" s="32">
+      <c r="D79" s="30">
         <v>5.0530101060202127E-3</v>
       </c>
     </row>
@@ -23178,7 +23180,7 @@
       <c r="C80" s="20">
         <v>1.006</v>
       </c>
-      <c r="D80" s="32">
+      <c r="D80" s="30">
         <v>5.0220100440200883E-3</v>
       </c>
     </row>
@@ -23192,7 +23194,7 @@
       <c r="C81" s="20">
         <v>1.0089999999999999</v>
       </c>
-      <c r="D81" s="32">
+      <c r="D81" s="30">
         <v>4.9600099200198368E-3</v>
       </c>
     </row>
@@ -23206,7 +23208,7 @@
       <c r="C82" s="20">
         <v>1.016</v>
       </c>
-      <c r="D82" s="32">
+      <c r="D82" s="30">
         <v>6.0450120900241815E-3</v>
       </c>
     </row>
@@ -23220,7 +23222,7 @@
       <c r="C83" s="20">
         <v>1.01</v>
       </c>
-      <c r="D83" s="32">
+      <c r="D83" s="30">
         <v>5.8280116560233131E-3</v>
       </c>
     </row>
@@ -23234,7 +23236,7 @@
       <c r="C84" s="20">
         <v>1.0209999999999999</v>
       </c>
-      <c r="D84" s="32">
+      <c r="D84" s="30">
         <v>6.045012090024178E-3</v>
       </c>
     </row>
@@ -23248,7 +23250,7 @@
       <c r="C85" s="20">
         <v>1.0369999999999999</v>
       </c>
-      <c r="D85" s="32">
+      <c r="D85" s="30">
         <v>5.98301196602393E-3</v>
       </c>
     </row>
@@ -23262,7 +23264,7 @@
       <c r="C86" s="20">
         <v>1.0389999999999999</v>
       </c>
-      <c r="D86" s="32">
+      <c r="D86" s="30">
         <v>5.8900117800235576E-3</v>
       </c>
     </row>
@@ -23276,7 +23278,7 @@
       <c r="C87" s="20">
         <v>1.042</v>
       </c>
-      <c r="D87" s="32">
+      <c r="D87" s="30">
         <v>6.8510137020274062E-3</v>
       </c>
     </row>
@@ -23290,7 +23292,7 @@
       <c r="C88" s="20">
         <v>1.032</v>
       </c>
-      <c r="D88" s="32">
+      <c r="D88" s="30">
         <v>6.5100130200260418E-3</v>
       </c>
     </row>
@@ -23304,7 +23306,7 @@
       <c r="C89" s="20">
         <v>1.044</v>
       </c>
-      <c r="D89" s="32">
+      <c r="D89" s="30">
         <v>6.7580135160270338E-3</v>
       </c>
     </row>
@@ -23318,7 +23320,7 @@
       <c r="C90" s="20">
         <v>1.06</v>
       </c>
-      <c r="D90" s="32">
+      <c r="D90" s="30">
         <v>6.6960133920267858E-3</v>
       </c>
     </row>
@@ -23332,7 +23334,7 @@
       <c r="C91" s="20">
         <v>1.0580000000000001</v>
       </c>
-      <c r="D91" s="32">
+      <c r="D91" s="30">
         <v>6.4790129580259174E-3</v>
       </c>
     </row>
@@ -23346,7 +23348,7 @@
       <c r="C92" s="20">
         <v>1.0529999999999999</v>
       </c>
-      <c r="D92" s="32">
+      <c r="D92" s="30">
         <v>7.1920143840287672E-3</v>
       </c>
     </row>
@@ -23360,7 +23362,7 @@
       <c r="C93" s="20">
         <v>1.044</v>
       </c>
-      <c r="D93" s="32">
+      <c r="D93" s="30">
         <v>6.8820137640275298E-3</v>
       </c>
     </row>
@@ -23374,7 +23376,7 @@
       <c r="C94" s="20">
         <v>1.0569999999999999</v>
       </c>
-      <c r="D94" s="32">
+      <c r="D94" s="30">
         <v>7.1610143220286427E-3</v>
       </c>
     </row>
@@ -23388,7 +23390,7 @@
       <c r="C95" s="20">
         <v>1.0680000000000001</v>
       </c>
-      <c r="D95" s="32">
+      <c r="D95" s="30">
         <v>6.9440138880277778E-3</v>
       </c>
     </row>
@@ -23402,7 +23404,7 @@
       <c r="C96" s="20">
         <v>1.079</v>
       </c>
-      <c r="D96" s="32">
+      <c r="D96" s="30">
         <v>7.1300142600285192E-3</v>
       </c>
     </row>
@@ -23416,7 +23418,7 @@
       <c r="C97" s="20">
         <v>1.0640000000000001</v>
       </c>
-      <c r="D97" s="32">
+      <c r="D97" s="30">
         <v>7.533015066030135E-3</v>
       </c>
     </row>
@@ -23430,7 +23432,7 @@
       <c r="C98" s="20">
         <v>1.0529999999999999</v>
       </c>
-      <c r="D98" s="32">
+      <c r="D98" s="30">
         <v>7.1610143220286427E-3</v>
       </c>
     </row>
@@ -23444,7 +23446,7 @@
       <c r="C99" s="20">
         <v>1.075</v>
       </c>
-      <c r="D99" s="32">
+      <c r="D99" s="30">
         <v>7.7190154380308755E-3</v>
       </c>
     </row>
@@ -23458,7 +23460,7 @@
       <c r="C100" s="20">
         <v>1.0860000000000001</v>
       </c>
-      <c r="D100" s="32">
+      <c r="D100" s="30">
         <v>7.5020150040300106E-3</v>
       </c>
     </row>
@@ -23472,7 +23474,7 @@
       <c r="C101" s="20">
         <v>1.091</v>
       </c>
-      <c r="D101" s="32">
+      <c r="D101" s="30">
         <v>7.5020150040300071E-3</v>
       </c>
     </row>
@@ -23486,7 +23488,7 @@
       <c r="C102" s="20">
         <v>1.0840000000000001</v>
       </c>
-      <c r="D102" s="32">
+      <c r="D102" s="30">
         <v>8.153016306032615E-3</v>
       </c>
     </row>
@@ -23500,7 +23502,7 @@
       <c r="C103" s="20">
         <v>1.069</v>
       </c>
-      <c r="D103" s="32">
+      <c r="D103" s="30">
         <v>7.6570153140306275E-3</v>
       </c>
     </row>
@@ -23514,7 +23516,7 @@
       <c r="C104" s="20">
         <v>1.091</v>
       </c>
-      <c r="D104" s="32">
+      <c r="D104" s="30">
         <v>8.2150164300328603E-3</v>
       </c>
     </row>
@@ -23528,7 +23530,7 @@
       <c r="C105" s="20">
         <v>1.093</v>
       </c>
-      <c r="D105" s="32">
+      <c r="D105" s="30">
         <v>7.7190154380308755E-3</v>
       </c>
     </row>
@@ -23542,7 +23544,7 @@
       <c r="C106" s="20">
         <v>1.103</v>
       </c>
-      <c r="D106" s="32">
+      <c r="D106" s="30">
         <v>7.874015748031496E-3</v>
       </c>
     </row>
@@ -23556,7 +23558,7 @@
       <c r="C107" s="20">
         <v>0.85799999999999998</v>
       </c>
-      <c r="D107" s="32">
+      <c r="D107" s="30">
         <v>0</v>
       </c>
     </row>
@@ -23570,7 +23572,7 @@
       <c r="C108" s="20">
         <v>0.83899999999999997</v>
       </c>
-      <c r="D108" s="32">
+      <c r="D108" s="30">
         <v>0</v>
       </c>
     </row>
@@ -23584,7 +23586,7 @@
       <c r="C109" s="20">
         <v>0.86399999999999999</v>
       </c>
-      <c r="D109" s="32">
+      <c r="D109" s="30">
         <v>0</v>
       </c>
     </row>
@@ -23598,7 +23600,7 @@
       <c r="C110" s="20">
         <v>0.85699999999999998</v>
       </c>
-      <c r="D110" s="32">
+      <c r="D110" s="30">
         <v>0</v>
       </c>
     </row>
@@ -23612,7 +23614,7 @@
       <c r="C111" s="20">
         <v>0.85799999999999998</v>
       </c>
-      <c r="D111" s="32">
+      <c r="D111" s="30">
         <v>0</v>
       </c>
     </row>
@@ -23626,7 +23628,7 @@
       <c r="C112" s="20">
         <v>1.0169999999999999</v>
       </c>
-      <c r="D112" s="32">
+      <c r="D112" s="30">
         <v>4.9290098580197133E-3</v>
       </c>
     </row>
@@ -23640,7 +23642,7 @@
       <c r="C113" s="20">
         <v>0.99399999999999999</v>
       </c>
-      <c r="D113" s="32">
+      <c r="D113" s="30">
         <v>4.8050096100192207E-3</v>
       </c>
     </row>
@@ -23654,7 +23656,7 @@
       <c r="C114" s="20">
         <v>1.0169999999999999</v>
       </c>
-      <c r="D114" s="32">
+      <c r="D114" s="30">
         <v>4.7430094860189693E-3</v>
       </c>
     </row>
@@ -23668,7 +23670,7 @@
       <c r="C115" s="20">
         <v>1.0169999999999999</v>
       </c>
-      <c r="D115" s="32">
+      <c r="D115" s="30">
         <v>4.9600099200198368E-3</v>
       </c>
     </row>
@@ -23682,7 +23684,7 @@
       <c r="C116" s="20">
         <v>1.026</v>
       </c>
-      <c r="D116" s="32">
+      <c r="D116" s="30">
         <v>5.2080104160208331E-3</v>
       </c>
     </row>
@@ -23696,7 +23698,7 @@
       <c r="C117" s="20">
         <v>1.032</v>
       </c>
-      <c r="D117" s="32">
+      <c r="D117" s="30">
         <v>5.3940107880215771E-3</v>
       </c>
     </row>
@@ -23710,7 +23712,7 @@
       <c r="C118" s="20">
         <v>1.0209999999999999</v>
       </c>
-      <c r="D118" s="32">
+      <c r="D118" s="30">
         <v>5.6420112840225656E-3</v>
       </c>
     </row>
@@ -23724,7 +23726,7 @@
       <c r="C119" s="20">
         <v>1.0429999999999999</v>
       </c>
-      <c r="D119" s="32">
+      <c r="D119" s="30">
         <v>5.5490110980221941E-3</v>
       </c>
     </row>
@@ -23738,7 +23740,7 @@
       <c r="C120" s="20">
         <v>1.0429999999999999</v>
       </c>
-      <c r="D120" s="32">
+      <c r="D120" s="30">
         <v>5.7660115320230616E-3</v>
       </c>
     </row>
@@ -23752,7 +23754,7 @@
       <c r="C121" s="20">
         <v>1.05</v>
       </c>
-      <c r="D121" s="32">
+      <c r="D121" s="30">
         <v>5.952011904023809E-3</v>
       </c>
     </row>
@@ -23766,7 +23768,7 @@
       <c r="C122" s="20">
         <v>1.0529999999999999</v>
       </c>
-      <c r="D122" s="32">
+      <c r="D122" s="30">
         <v>6.045012090024178E-3</v>
       </c>
     </row>
@@ -23780,7 +23782,7 @@
       <c r="C123" s="20">
         <v>1.0329999999999999</v>
       </c>
-      <c r="D123" s="32">
+      <c r="D123" s="30">
         <v>6.0140120280240544E-3</v>
       </c>
     </row>
@@ -23794,7 +23796,7 @@
       <c r="C124" s="20">
         <v>1.0640000000000001</v>
       </c>
-      <c r="D124" s="32">
+      <c r="D124" s="30">
         <v>6.2000124000248019E-3</v>
       </c>
     </row>
@@ -23808,7 +23810,7 @@
       <c r="C125" s="20">
         <v>1.0589999999999999</v>
       </c>
-      <c r="D125" s="32">
+      <c r="D125" s="30">
         <v>6.2620125240250464E-3</v>
       </c>
     </row>
@@ -23822,7 +23824,7 @@
       <c r="C126" s="20">
         <v>1.0760000000000001</v>
       </c>
-      <c r="D126" s="32">
+      <c r="D126" s="30">
         <v>6.7580135160270338E-3</v>
       </c>
     </row>
@@ -23836,7 +23838,7 @@
       <c r="C127" s="20">
         <v>1.0660000000000001</v>
       </c>
-      <c r="D127" s="32">
+      <c r="D127" s="30">
         <v>6.4480128960257939E-3</v>
       </c>
     </row>
@@ -23850,7 +23852,7 @@
       <c r="C128" s="20">
         <v>1.0609999999999999</v>
       </c>
-      <c r="D128" s="32">
+      <c r="D128" s="30">
         <v>6.8820137640275263E-3</v>
       </c>
     </row>
@@ -23864,7 +23866,7 @@
       <c r="C129" s="20">
         <v>1.075</v>
       </c>
-      <c r="D129" s="32">
+      <c r="D129" s="30">
         <v>6.5410130820261628E-3</v>
       </c>
     </row>
@@ -23878,7 +23880,7 @@
       <c r="C130" s="20">
         <v>1.075</v>
       </c>
-      <c r="D130" s="32">
+      <c r="D130" s="30">
         <v>6.7580135160270303E-3</v>
       </c>
     </row>
@@ -23892,7 +23894,7 @@
       <c r="C131" s="20">
         <v>1.0960000000000001</v>
       </c>
-      <c r="D131" s="32">
+      <c r="D131" s="30">
         <v>7.3780147560295146E-3</v>
       </c>
     </row>
@@ -23906,7 +23908,7 @@
       <c r="C132" s="20">
         <v>1.079</v>
       </c>
-      <c r="D132" s="32">
+      <c r="D132" s="30">
         <v>6.8510137020274028E-3</v>
       </c>
     </row>
@@ -23920,7 +23922,7 @@
       <c r="C133" s="20">
         <v>1.0620000000000001</v>
       </c>
-      <c r="D133" s="32">
+      <c r="D133" s="30">
         <v>6.9130138260276542E-3</v>
       </c>
     </row>
@@ -23934,7 +23936,7 @@
       <c r="C134" s="20">
         <v>1.0880000000000001</v>
       </c>
-      <c r="D134" s="32">
+      <c r="D134" s="30">
         <v>6.9440138880277778E-3</v>
       </c>
     </row>
@@ -23948,7 +23950,7 @@
       <c r="C135" s="20">
         <v>1.1040000000000001</v>
       </c>
-      <c r="D135" s="32">
+      <c r="D135" s="30">
         <v>7.657015314030631E-3</v>
       </c>
     </row>
@@ -23962,7 +23964,7 @@
       <c r="C136" s="20">
         <v>1.1240000000000001</v>
       </c>
-      <c r="D136" s="32">
+      <c r="D136" s="30">
         <v>8.2460164920329874E-3</v>
       </c>
     </row>
@@ -23976,7 +23978,7 @@
       <c r="C137" s="20">
         <v>1.0880000000000001</v>
       </c>
-      <c r="D137" s="32">
+      <c r="D137" s="30">
         <v>7.1300142600285226E-3</v>
       </c>
     </row>
@@ -23990,7 +23992,7 @@
       <c r="C138" s="20">
         <v>1.0860000000000001</v>
       </c>
-      <c r="D138" s="32">
+      <c r="D138" s="30">
         <v>7.657015314030631E-3</v>
       </c>
     </row>
@@ -24004,7 +24006,7 @@
       <c r="C139" s="20">
         <v>1.105</v>
       </c>
-      <c r="D139" s="32">
+      <c r="D139" s="30">
         <v>7.4710149420298836E-3</v>
       </c>
     </row>
@@ -24018,7 +24020,7 @@
       <c r="C140" s="20">
         <v>1.113</v>
       </c>
-      <c r="D140" s="32">
+      <c r="D140" s="30">
         <v>7.9360158720317431E-3</v>
       </c>
     </row>
@@ -24032,7 +24034,7 @@
       <c r="C141" s="20">
         <v>1.113</v>
       </c>
-      <c r="D141" s="32">
+      <c r="D141" s="30">
         <v>7.9050158100316195E-3</v>
       </c>
     </row>
@@ -24046,7 +24048,7 @@
       <c r="C142" s="20">
         <v>0.85799999999999998</v>
       </c>
-      <c r="D142" s="32">
+      <c r="D142" s="30">
         <v>0</v>
       </c>
     </row>
@@ -24060,7 +24062,7 @@
       <c r="C143" s="20">
         <v>0.84</v>
       </c>
-      <c r="D143" s="32">
+      <c r="D143" s="30">
         <v>0</v>
       </c>
     </row>
@@ -24074,7 +24076,7 @@
       <c r="C144" s="20">
         <v>0.83199999999999996</v>
       </c>
-      <c r="D144" s="32">
+      <c r="D144" s="30">
         <v>0</v>
       </c>
     </row>
@@ -24088,7 +24090,7 @@
       <c r="C145" s="20">
         <v>0.84899999999999998</v>
       </c>
-      <c r="D145" s="32">
+      <c r="D145" s="30">
         <v>0</v>
       </c>
     </row>
@@ -24102,7 +24104,7 @@
       <c r="C146" s="20">
         <v>0.84699999999999998</v>
       </c>
-      <c r="D146" s="32">
+      <c r="D146" s="30">
         <v>0</v>
       </c>
     </row>
@@ -24116,7 +24118,7 @@
       <c r="C147" s="20">
         <v>1.0289999999999999</v>
       </c>
-      <c r="D147" s="32">
+      <c r="D147" s="30">
         <v>5.3010106020212012E-3</v>
       </c>
     </row>
@@ -24130,7 +24132,7 @@
       <c r="C148" s="20">
         <v>1.0129999999999999</v>
       </c>
-      <c r="D148" s="32">
+      <c r="D148" s="30">
         <v>5.3630107260214492E-3</v>
       </c>
     </row>
@@ -24144,7 +24146,7 @@
       <c r="C149" s="20">
         <v>1.0129999999999999</v>
       </c>
-      <c r="D149" s="32">
+      <c r="D149" s="30">
         <v>5.611011222022442E-3</v>
       </c>
     </row>
@@ -24158,7 +24160,7 @@
       <c r="C150" s="20">
         <v>1.034</v>
       </c>
-      <c r="D150" s="32">
+      <c r="D150" s="30">
         <v>5.7350114700229415E-3</v>
       </c>
     </row>
@@ -24172,7 +24174,7 @@
       <c r="C151" s="20">
         <v>1.0109999999999999</v>
       </c>
-      <c r="D151" s="32">
+      <c r="D151" s="30">
         <v>5.0840101680203337E-3</v>
       </c>
     </row>
@@ -24186,7 +24188,7 @@
       <c r="C152" s="20">
         <v>1.056</v>
       </c>
-      <c r="D152" s="32">
+      <c r="D152" s="30">
         <v>6.1380122760245539E-3</v>
       </c>
     </row>
@@ -24200,7 +24202,7 @@
       <c r="C153" s="20">
         <v>1.034</v>
       </c>
-      <c r="D153" s="32">
+      <c r="D153" s="30">
         <v>6.014012028024057E-3</v>
       </c>
     </row>
@@ -24214,7 +24216,7 @@
       <c r="C154" s="20">
         <v>1.0429999999999999</v>
       </c>
-      <c r="D154" s="32">
+      <c r="D154" s="30">
         <v>6.5410130820261628E-3</v>
       </c>
     </row>
@@ -24228,7 +24230,7 @@
       <c r="C155" s="20">
         <v>1.0580000000000001</v>
       </c>
-      <c r="D155" s="32">
+      <c r="D155" s="30">
         <v>6.4790129580259174E-3</v>
       </c>
     </row>
@@ -24242,7 +24244,7 @@
       <c r="C156" s="20">
         <v>1.05</v>
       </c>
-      <c r="D156" s="32">
+      <c r="D156" s="30">
         <v>6.2930125860251734E-3</v>
       </c>
     </row>
@@ -24256,7 +24258,7 @@
       <c r="C157" s="20">
         <v>1.0740000000000001</v>
       </c>
-      <c r="D157" s="32">
+      <c r="D157" s="30">
         <v>6.6960133920267858E-3</v>
       </c>
     </row>
@@ -24270,7 +24272,7 @@
       <c r="C158" s="20">
         <v>1.0629999999999999</v>
       </c>
-      <c r="D158" s="32">
+      <c r="D158" s="30">
         <v>6.9130138260276508E-3</v>
       </c>
     </row>
@@ -24284,7 +24286,7 @@
       <c r="C159" s="20">
         <v>1.075</v>
       </c>
-      <c r="D159" s="32">
+      <c r="D159" s="30">
         <v>7.5330150660301316E-3</v>
       </c>
     </row>
@@ -24298,7 +24300,7 @@
       <c r="C160" s="20">
         <v>1.0860000000000001</v>
       </c>
-      <c r="D160" s="32">
+      <c r="D160" s="30">
         <v>7.3470146940293902E-3</v>
       </c>
     </row>
@@ -24312,7 +24314,7 @@
       <c r="C161" s="20">
         <v>1.0720000000000001</v>
       </c>
-      <c r="D161" s="32">
+      <c r="D161" s="30">
         <v>6.9750139500279022E-3</v>
       </c>
     </row>
@@ -24326,7 +24328,7 @@
       <c r="C162" s="20">
         <v>1.099</v>
       </c>
-      <c r="D162" s="32">
+      <c r="D162" s="30">
         <v>7.4710149420298836E-3</v>
       </c>
     </row>
@@ -24340,7 +24342,7 @@
       <c r="C163" s="20">
         <v>1.083</v>
       </c>
-      <c r="D163" s="32">
+      <c r="D163" s="30">
         <v>7.5330150660301316E-3</v>
       </c>
     </row>
@@ -24354,7 +24356,7 @@
       <c r="C164" s="20">
         <v>1.087</v>
       </c>
-      <c r="D164" s="32">
+      <c r="D164" s="30">
         <v>7.9050158100316195E-3</v>
       </c>
     </row>
@@ -24368,7 +24370,7 @@
       <c r="C165" s="20">
         <v>1.109</v>
       </c>
-      <c r="D165" s="32">
+      <c r="D165" s="30">
         <v>8.0600161200322391E-3</v>
       </c>
     </row>
@@ -24382,7 +24384,7 @@
       <c r="C166" s="20">
         <v>1.099</v>
       </c>
-      <c r="D166" s="32">
+      <c r="D166" s="30">
         <v>7.8120156240312471E-3</v>
       </c>
     </row>
@@ -24396,7 +24398,7 @@
       <c r="C167" s="20">
         <v>1.1080000000000001</v>
       </c>
-      <c r="D167" s="32">
+      <c r="D167" s="30">
         <v>7.7500155000310026E-3</v>
       </c>
     </row>
@@ -24410,7 +24412,7 @@
       <c r="C168" s="20">
         <v>1.089</v>
       </c>
-      <c r="D168" s="32">
+      <c r="D168" s="30">
         <v>7.7190154380308755E-3</v>
       </c>
     </row>
@@ -24424,7 +24426,7 @@
       <c r="C169" s="20">
         <v>1.1020000000000001</v>
       </c>
-      <c r="D169" s="32">
+      <c r="D169" s="30">
         <v>8.3700167400334834E-3</v>
       </c>
     </row>
@@ -24438,7 +24440,7 @@
       <c r="C170" s="20">
         <v>1.125</v>
       </c>
-      <c r="D170" s="32">
+      <c r="D170" s="30">
         <v>8.5560171120342247E-3</v>
       </c>
     </row>
@@ -24452,7 +24454,7 @@
       <c r="C171" s="20">
         <v>1.1100000000000001</v>
       </c>
-      <c r="D171" s="32">
+      <c r="D171" s="30">
         <v>8.153016306032615E-3</v>
       </c>
     </row>
@@ -24466,7 +24468,7 @@
       <c r="C172" s="20">
         <v>1.1200000000000001</v>
       </c>
-      <c r="D172" s="32">
+      <c r="D172" s="30">
         <v>8.1220162440324914E-3</v>
       </c>
     </row>
@@ -24480,7 +24482,7 @@
       <c r="C173" s="20">
         <v>1.1000000000000001</v>
       </c>
-      <c r="D173" s="32">
+      <c r="D173" s="30">
         <v>8.0600161200322425E-3</v>
       </c>
     </row>
@@ -24494,7 +24496,7 @@
       <c r="C174" s="20">
         <v>1.115</v>
       </c>
-      <c r="D174" s="32">
+      <c r="D174" s="30">
         <v>8.7730175460350914E-3</v>
       </c>
     </row>
@@ -24508,7 +24510,7 @@
       <c r="C175" s="20">
         <v>1.145</v>
       </c>
-      <c r="D175" s="32">
+      <c r="D175" s="30">
         <v>9.1760183520367047E-3</v>
       </c>
     </row>
@@ -24522,7 +24524,7 @@
       <c r="C176" s="20">
         <v>1.1259999999999999</v>
       </c>
-      <c r="D176" s="32">
+      <c r="D176" s="30">
         <v>8.649017298034592E-3</v>
       </c>
     </row>
@@ -24536,7 +24538,7 @@
       <c r="C177" s="20">
         <v>0.873</v>
       </c>
-      <c r="D177" s="32">
+      <c r="D177" s="30">
         <v>0</v>
       </c>
     </row>
@@ -24550,7 +24552,7 @@
       <c r="C178" s="20">
         <v>0.874</v>
       </c>
-      <c r="D178" s="32">
+      <c r="D178" s="30">
         <v>0</v>
       </c>
     </row>
@@ -24564,7 +24566,7 @@
       <c r="C179" s="20">
         <v>0.88900000000000001</v>
       </c>
-      <c r="D179" s="32">
+      <c r="D179" s="30">
         <v>0</v>
       </c>
     </row>
@@ -24578,7 +24580,7 @@
       <c r="C180" s="20">
         <v>0.90900000000000003</v>
       </c>
-      <c r="D180" s="32">
+      <c r="D180" s="30">
         <v>0</v>
       </c>
     </row>
@@ -24592,7 +24594,7 @@
       <c r="C181" s="20">
         <v>0.88</v>
       </c>
-      <c r="D181" s="32">
+      <c r="D181" s="30">
         <v>0</v>
       </c>
     </row>
@@ -24606,7 +24608,7 @@
       <c r="C182" s="20">
         <v>0.97599999999999998</v>
       </c>
-      <c r="D182" s="32">
+      <c r="D182" s="30">
         <v>3.1930063860127712E-3</v>
       </c>
     </row>
@@ -24620,7 +24622,7 @@
       <c r="C183" s="20">
         <v>0.97299999999999998</v>
       </c>
-      <c r="D183" s="32">
+      <c r="D183" s="30">
         <v>3.0690061380122752E-3</v>
       </c>
     </row>
@@ -24634,7 +24636,7 @@
       <c r="C184" s="20">
         <v>0.98699999999999999</v>
       </c>
-      <c r="D184" s="32">
+      <c r="D184" s="30">
         <v>3.0380060760121512E-3</v>
       </c>
     </row>
@@ -24648,7 +24650,7 @@
       <c r="C185" s="20">
         <v>1.012</v>
       </c>
-      <c r="D185" s="32">
+      <c r="D185" s="30">
         <v>3.1930063860127712E-3</v>
       </c>
     </row>
@@ -24662,7 +24664,7 @@
       <c r="C186" s="20">
         <v>0.97</v>
       </c>
-      <c r="D186" s="32">
+      <c r="D186" s="30">
         <v>2.7900055800111588E-3</v>
       </c>
     </row>
@@ -24676,7 +24678,7 @@
       <c r="C187" s="20">
         <v>1.014</v>
       </c>
-      <c r="D187" s="32">
+      <c r="D187" s="30">
         <v>4.3710087420174839E-3</v>
       </c>
     </row>
@@ -24690,7 +24692,7 @@
       <c r="C188" s="20">
         <v>1.0089999999999999</v>
       </c>
-      <c r="D188" s="32">
+      <c r="D188" s="30">
         <v>4.1850083700167365E-3</v>
       </c>
     </row>
@@ -24704,7 +24706,7 @@
       <c r="C189" s="20">
         <v>1.028</v>
       </c>
-      <c r="D189" s="32">
+      <c r="D189" s="30">
         <v>4.3090086180172359E-3</v>
       </c>
     </row>
@@ -24718,7 +24720,7 @@
       <c r="C190" s="20">
         <v>1.0609999999999999</v>
       </c>
-      <c r="D190" s="32">
+      <c r="D190" s="30">
         <v>4.7120094240188449E-3</v>
       </c>
     </row>
@@ -24732,7 +24734,7 @@
       <c r="C191" s="20">
         <v>1.0169999999999999</v>
       </c>
-      <c r="D191" s="32">
+      <c r="D191" s="30">
         <v>4.2470084940169845E-3</v>
       </c>
     </row>
@@ -24746,7 +24748,7 @@
       <c r="C192" s="20">
         <v>1.0369999999999999</v>
       </c>
-      <c r="D192" s="32">
+      <c r="D192" s="30">
         <v>5.0840101680203337E-3</v>
       </c>
     </row>
@@ -24760,7 +24762,7 @@
       <c r="C193" s="20">
         <v>1.0269999999999999</v>
       </c>
-      <c r="D193" s="32">
+      <c r="D193" s="30">
         <v>4.7430094860189693E-3</v>
       </c>
     </row>
@@ -24774,7 +24776,7 @@
       <c r="C194" s="20">
         <v>1.0580000000000001</v>
       </c>
-      <c r="D194" s="32">
+      <c r="D194" s="30">
         <v>5.2390104780209567E-3</v>
       </c>
     </row>
@@ -24788,7 +24790,7 @@
       <c r="C195" s="20">
         <v>1.1000000000000001</v>
       </c>
-      <c r="D195" s="32">
+      <c r="D195" s="30">
         <v>5.9210118420236855E-3</v>
       </c>
     </row>
@@ -24802,7 +24804,7 @@
       <c r="C196" s="20">
         <v>1.056</v>
       </c>
-      <c r="D196" s="32">
+      <c r="D196" s="30">
         <v>5.4560109120218251E-3</v>
       </c>
     </row>
@@ -24816,7 +24818,7 @@
       <c r="C197" s="20">
         <v>1.056</v>
       </c>
-      <c r="D197" s="32">
+      <c r="D197" s="30">
         <v>5.6730113460226935E-3</v>
       </c>
     </row>
@@ -24830,7 +24832,7 @@
       <c r="C198" s="20">
         <v>1.044</v>
       </c>
-      <c r="D198" s="32">
+      <c r="D198" s="30">
         <v>5.2700105400210811E-3</v>
       </c>
     </row>
@@ -24844,7 +24846,7 @@
       <c r="C199" s="20">
         <v>1.0840000000000001</v>
       </c>
-      <c r="D199" s="32">
+      <c r="D199" s="30">
         <v>6.0450120900241815E-3</v>
       </c>
     </row>
@@ -24858,7 +24860,7 @@
       <c r="C200" s="20">
         <v>1.135</v>
       </c>
-      <c r="D200" s="32">
+      <c r="D200" s="30">
         <v>7.0060140120280232E-3</v>
       </c>
     </row>
@@ -24872,7 +24874,7 @@
       <c r="C201" s="20">
         <v>1.0840000000000001</v>
       </c>
-      <c r="D201" s="32">
+      <c r="D201" s="30">
         <v>6.3240126480252979E-3</v>
       </c>
     </row>
@@ -24886,7 +24888,7 @@
       <c r="C202" s="20">
         <v>1.079</v>
       </c>
-      <c r="D202" s="32">
+      <c r="D202" s="30">
         <v>6.3860127720255424E-3</v>
       </c>
     </row>
@@ -24900,7 +24902,7 @@
       <c r="C203" s="20">
         <v>1.0640000000000001</v>
       </c>
-      <c r="D203" s="32">
+      <c r="D203" s="30">
         <v>5.8900117800235611E-3</v>
       </c>
     </row>
@@ -24914,7 +24916,7 @@
       <c r="C204" s="20">
         <v>1.107</v>
       </c>
-      <c r="D204" s="32">
+      <c r="D204" s="30">
         <v>6.7580135160270303E-3</v>
       </c>
     </row>
@@ -24928,7 +24930,7 @@
       <c r="C205" s="20">
         <v>1.17</v>
       </c>
-      <c r="D205" s="32">
+      <c r="D205" s="30">
         <v>8.0910161820323609E-3</v>
       </c>
     </row>
@@ -24942,7 +24944,7 @@
       <c r="C206" s="20">
         <v>1.117</v>
       </c>
-      <c r="D206" s="32">
+      <c r="D206" s="30">
         <v>7.3470146940293867E-3</v>
       </c>
     </row>
@@ -24956,7 +24958,7 @@
       <c r="C207" s="20">
         <v>1.0940000000000001</v>
       </c>
-      <c r="D207" s="32">
+      <c r="D207" s="30">
         <v>6.8510137020274062E-3</v>
       </c>
     </row>
@@ -24970,7 +24972,7 @@
       <c r="C208" s="20">
         <v>1.085</v>
       </c>
-      <c r="D208" s="32">
+      <c r="D208" s="30">
         <v>6.5410130820261628E-3</v>
       </c>
     </row>
@@ -24984,7 +24986,7 @@
       <c r="C209" s="20">
         <v>1.1299999999999999</v>
       </c>
-      <c r="D209" s="32">
+      <c r="D209" s="30">
         <v>7.4710149420298801E-3</v>
       </c>
     </row>
@@ -24998,7 +25000,7 @@
       <c r="C210" s="20">
         <v>1.208</v>
       </c>
-      <c r="D210" s="32">
+      <c r="D210" s="30">
         <v>9.2690185380370736E-3</v>
       </c>
     </row>
@@ -25012,7 +25014,7 @@
       <c r="C211" s="20">
         <v>1.1499999999999999</v>
       </c>
-      <c r="D211" s="32">
+      <c r="D211" s="30">
         <v>8.3700167400334764E-3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
working on tensile index results
</commit_message>
<xml_diff>
--- a/IP_Absorption.xlsx
+++ b/IP_Absorption.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="277" documentId="8_{D2BF99F2-6939-1445-9333-69AF606EB5C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBE1EDA3-0506-C34B-9FD5-F9BFC4B63900}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="15620" windowHeight="17180" activeTab="2" xr2:uid="{E0E81384-8338-6A40-B1D6-6AC1A920927D}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="19780" windowHeight="17180" activeTab="2" xr2:uid="{E0E81384-8338-6A40-B1D6-6AC1A920927D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -302,13 +302,13 @@
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15160,24 +15160,24 @@
       <c r="P44" s="4"/>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A45" s="31" t="s">
+      <c r="A45" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="B45" s="31"/>
-      <c r="C45" s="31"/>
-      <c r="D45" s="31"/>
-      <c r="E45" s="31"/>
-      <c r="F45" s="31"/>
-      <c r="G45" s="31"/>
-      <c r="H45" s="31"/>
-      <c r="I45" s="31"/>
-      <c r="J45" s="31"/>
-      <c r="K45" s="31"/>
-      <c r="L45" s="31"/>
-      <c r="M45" s="31"/>
-      <c r="N45" s="31"/>
-      <c r="O45" s="31"/>
-      <c r="P45" s="31"/>
+      <c r="B45" s="32"/>
+      <c r="C45" s="32"/>
+      <c r="D45" s="32"/>
+      <c r="E45" s="32"/>
+      <c r="F45" s="32"/>
+      <c r="G45" s="32"/>
+      <c r="H45" s="32"/>
+      <c r="I45" s="32"/>
+      <c r="J45" s="32"/>
+      <c r="K45" s="32"/>
+      <c r="L45" s="32"/>
+      <c r="M45" s="32"/>
+      <c r="N45" s="32"/>
+      <c r="O45" s="32"/>
+      <c r="P45" s="32"/>
     </row>
     <row r="46" spans="1:16" ht="51" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
@@ -18284,13 +18284,13 @@
       <c r="F1" s="2"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
       <c r="F2" s="1"/>
     </row>
     <row r="3" spans="1:8" ht="51" x14ac:dyDescent="0.2">
@@ -19342,13 +19342,13 @@
       <c r="F52" s="4"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A53" s="31" t="s">
+      <c r="A53" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="B53" s="31"/>
-      <c r="C53" s="31"/>
-      <c r="D53" s="31"/>
-      <c r="E53" s="31"/>
+      <c r="B53" s="32"/>
+      <c r="C53" s="32"/>
+      <c r="D53" s="32"/>
+      <c r="E53" s="32"/>
       <c r="F53" s="1"/>
     </row>
     <row r="54" spans="1:8" ht="51" x14ac:dyDescent="0.2">
@@ -22146,7 +22146,7 @@
       <c r="D6" s="30">
         <v>0</v>
       </c>
-      <c r="F6" s="33"/>
+      <c r="F6" s="31"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="27">

</xml_diff>